<commit_message>
Batch 2026-10: production database verify passed — F14.2.1 DONE in tracker and report
Verify run 39211030047 (19 Oct) passed after the owner added
PROD_DATABASE_HOST / PROD_DATABASE_NAME to the production environment:
database neondb on the production Neon host, 86 migrations, newest 0084 =
the release, none missing.

- Tracker: F14.2.1 DONE; F14.1.3 note updated.
- Testing report (md/html/pdf): production evidence and sign-off updated; the
  open "verify cannot run" item closed.
- Decision log D-R07; Owner inputs §13 marked done.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FQWm4cqibRLpvtz1hvkLto
</commit_message>
<xml_diff>
--- a/docs/gokesari-audit/GOKESARI_FEATURE_STATUS_REPORT_2026-10-18_batch.xlsx
+++ b/docs/gokesari-audit/GOKESARI_FEATURE_STATUS_REPORT_2026-10-18_batch.xlsx
@@ -2978,7 +2978,7 @@
       </c>
       <c r="E23" s="23" t="inlineStr">
         <is>
-          <t>Released to gokesari.com by #194 (merge fc70223, 20:45:32 UTC = restore point). Automated: 283/283 batch cases + 8 mobile; whole suite 2191/2192 (1 pre-existing load flake); CI green on #190/#192/#193/#194. test.gokesari.com: remote checks 12/12; signed-in journeys 40 pass, 1 blocked (S-014 no rider online). gokesari.com: production-safe checks 12/12. Report: docs/test-reports/2026-10-batch.md. Production order lifecycle needs owner inputs §14.</t>
+          <t>Released to gokesari.com by #194 (merge fc70223, 20:45:32 UTC = restore point). Automated: 283/283 batch cases + 8 mobile; whole suite 2191/2192 (1 pre-existing load flake); CI green on #190/#192/#193/#194. test.gokesari.com: remote checks 12/12; signed-in journeys 40 pass, 1 blocked (S-014 no rider online). gokesari.com: production-safe checks 12/12; Production database verify passed (run 39211030047, 19 Oct: 0079–0084 applied, none missing). Report: docs/test-reports/2026-10-batch.md. Production order lifecycle needs owner inputs §14.</t>
         </is>
       </c>
     </row>
@@ -2993,9 +2993,9 @@
           <t>Migrate production through the 'Production database' workflow</t>
         </is>
       </c>
-      <c r="C24" s="41" t="inlineStr">
-        <is>
-          <t>BLOCKED-OWNER-INPUT</t>
+      <c r="C24" s="37" t="inlineStr">
+        <is>
+          <t>DONE</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -3005,7 +3005,7 @@
       </c>
       <c r="E24" s="23" t="inlineStr">
         <is>
-          <t>Fixed and released (#190, #194): the job now declares environment: production and a fail-fast preflight that lists what it can see without printing values. Production run 39165658144 (18 Oct, after the release) proves the fix for the secret: PROD_DATABASE_URL is now visible (it was empty on 15 Oct). It stops before touching production because the variables PROD_DATABASE_HOST and PROD_DATABASE_NAME are empty on the production environment — owner to add them (Owner inputs §13), then run verify.</t>
+          <t>Fixed and released (#190, #194): the job declares environment: production and a fail-fast preflight that lists what it can see without printing values. The owner added PROD_DATABASE_HOST / PROD_DATABASE_NAME to the production environment on 19 Oct (the values had been on an unused 'PROD' environment). Verify run 39211030047 (19 Oct) PASSED: all values visible, guard confirmed database neondb on the production Neon host, 86 migrations recorded, newest 0084_batch_f_notifications = release, none missing.</t>
         </is>
       </c>
     </row>
@@ -38697,7 +38697,7 @@
       </c>
       <c r="I200" s="12" t="inlineStr">
         <is>
-          <t>BLOCKED-OWNER-INPUT (18 Oct batch): Released to gokesari.com by #194 (merge fc70223, 20:45:32 UTC = restore point). Automated: 283/283 batch cases + 8 mobile; whole suite 2191/2192 (1 pre-existing load flake); CI green on #190/#192/#193/#194. test.gokesari.com: remote checks 12/12; signed-in journeys 40 pass, 1 blocked (S-014 no rider online). gokesari.com: production-safe checks 12/12. Report: docs/test-reports/2026-10-batch.md. Production order lifecycle needs owner inputs §14.</t>
+          <t>BLOCKED-OWNER-INPUT (18 Oct batch): Released to gokesari.com by #194 (merge fc70223, 20:45:32 UTC = restore point). Automated: 283/283 batch cases + 8 mobile; whole suite 2191/2192 (1 pre-existing load flake); CI green on #190/#192/#193/#194. test.gokesari.com: remote checks 12/12; signed-in journeys 40 pass, 1 blocked (S-014 no rider online). gokesari.com: production-safe checks 12/12; Production database verify passed (run 39211030047, 19 Oct: 0079–0084 applied, none missing). Report: docs/test-reports/2026-10-batch.md. Production order lifecycle needs owner inputs §14.</t>
         </is>
       </c>
       <c r="J200" s="41" t="inlineStr">
@@ -38712,7 +38712,7 @@
       </c>
       <c r="L200" s="23" t="inlineStr">
         <is>
-          <t>Released to gokesari.com by #194 (merge fc70223, 20:45:32 UTC = restore point). Automated: 283/283 batch cases + 8 mobile; whole suite 2191/2192 (1 pre-existing load flake); CI green on #190/#192/#193/#194. test.gokesari.com: remote checks 12/12; signed-in journeys 40 pass, 1 blocked (S-014 no rider online). gokesari.com: production-safe checks 12/12. Report: docs/test-reports/2026-10-batch.md. Production order lifecycle needs owner inputs §14.</t>
+          <t>Released to gokesari.com by #194 (merge fc70223, 20:45:32 UTC = restore point). Automated: 283/283 batch cases + 8 mobile; whole suite 2191/2192 (1 pre-existing load flake); CI green on #190/#192/#193/#194. test.gokesari.com: remote checks 12/12; signed-in journeys 40 pass, 1 blocked (S-014 no rider online). gokesari.com: production-safe checks 12/12; Production database verify passed (run 39211030047, 19 Oct: 0079–0084 applied, none missing). Report: docs/test-reports/2026-10-batch.md. Production order lifecycle needs owner inputs §14.</t>
         </is>
       </c>
     </row>
@@ -38856,7 +38856,7 @@
       <c r="F204" s="10" t="n"/>
       <c r="G204" s="10" t="inlineStr">
         <is>
-          <t>BLOCKED</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="H204" s="12" t="inlineStr">
@@ -38866,12 +38866,12 @@
       </c>
       <c r="I204" s="12" t="inlineStr">
         <is>
-          <t>BLOCKED-OWNER-INPUT (18 Oct batch): Fixed and released (#190, #194): the job now declares environment: production and a fail-fast preflight that lists what it can see without printing values. Production run 39165658144 (18 Oct, after the release) proves the fix for the secret: PROD_DATABASE_URL is now visible (it was empty on 15 Oct). It stops before touching production because the variables PROD_DATABASE_HOST and PROD_DATABASE_NAME are empty on the production environment — owner to add them (Owner inputs §13), then run verify.</t>
-        </is>
-      </c>
-      <c r="J204" s="41" t="inlineStr">
-        <is>
-          <t>BLOCKED-OWNER-INPUT</t>
+          <t>DONE (18 Oct batch): Fixed and released (#190, #194): the job declares environment: production and a fail-fast preflight that lists what it can see without printing values. The owner added PROD_DATABASE_HOST / PROD_DATABASE_NAME to the production environment on 19 Oct (the values had been on an unused 'PROD' environment). Verify run 39211030047 (19 Oct) PASSED: all values visible, guard confirmed database neondb on the production Neon host, 86 migrations recorded, newest 0084_batch_f_notifications = release, none missing.</t>
+        </is>
+      </c>
+      <c r="J204" s="37" t="inlineStr">
+        <is>
+          <t>DONE</t>
         </is>
       </c>
       <c r="K204" t="inlineStr">
@@ -38881,7 +38881,7 @@
       </c>
       <c r="L204" s="23" t="inlineStr">
         <is>
-          <t>Fixed and released (#190, #194): the job now declares environment: production and a fail-fast preflight that lists what it can see without printing values. Production run 39165658144 (18 Oct, after the release) proves the fix for the secret: PROD_DATABASE_URL is now visible (it was empty on 15 Oct). It stops before touching production because the variables PROD_DATABASE_HOST and PROD_DATABASE_NAME are empty on the production environment — owner to add them (Owner inputs §13), then run verify.</t>
+          <t>Fixed and released (#190, #194): the job declares environment: production and a fail-fast preflight that lists what it can see without printing values. The owner added PROD_DATABASE_HOST / PROD_DATABASE_NAME to the production environment on 19 Oct (the values had been on an unused 'PROD' environment). Verify run 39211030047 (19 Oct) PASSED: all values visible, guard confirmed database neondb on the production Neon host, 86 migrations recorded, newest 0084_batch_f_notifications = release, none missing.</t>
         </is>
       </c>
     </row>

</xml_diff>